<commit_message>
Logic: enabling works start after the HCIS documents (FS) at every station; construction follows enabling
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DZdGPWRxvKXCnMyT6qFPZb
</commit_message>
<xml_diff>
--- a/p6/0580_BOQ_Cost_Mapping.xlsx
+++ b/p6/0580_BOQ_Cost_Mapping.xlsx
@@ -2525,7 +2525,7 @@
     <row r="79">
       <c r="A79" s="8" t="inlineStr">
         <is>
-          <t>PRJ-M1150</t>
+          <t>NRY-E1120</t>
         </is>
       </c>
       <c r="B79" s="8" t="inlineStr">
@@ -2539,7 +2539,7 @@
         </is>
       </c>
       <c r="D79" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80">
@@ -3645,7 +3645,7 @@
     <row r="135">
       <c r="A135" s="8" t="inlineStr">
         <is>
-          <t>PRJ-M1150</t>
+          <t>HMK-E1120</t>
         </is>
       </c>
       <c r="B135" s="8" t="inlineStr">
@@ -3659,7 +3659,7 @@
         </is>
       </c>
       <c r="D135" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="136">
@@ -4685,7 +4685,7 @@
     <row r="187">
       <c r="A187" s="8" t="inlineStr">
         <is>
-          <t>ERY-E1010</t>
+          <t>ERY-E1120</t>
         </is>
       </c>
       <c r="B187" s="8" t="inlineStr">
@@ -4695,11 +4695,11 @@
       </c>
       <c r="C187" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D187" s="8" t="n">
-        <v>40</v>
+        <v>0</v>
       </c>
     </row>
     <row r="188">
@@ -5925,7 +5925,7 @@
     <row r="249">
       <c r="A249" s="8" t="inlineStr">
         <is>
-          <t>HJD-E1010</t>
+          <t>HJD-E1120</t>
         </is>
       </c>
       <c r="B249" s="8" t="inlineStr">
@@ -5935,11 +5935,11 @@
       </c>
       <c r="C249" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D249" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="250">
@@ -7165,7 +7165,7 @@
     <row r="311">
       <c r="A311" s="8" t="inlineStr">
         <is>
-          <t>EDM-E1010</t>
+          <t>EDM-E1120</t>
         </is>
       </c>
       <c r="B311" s="8" t="inlineStr">
@@ -7175,11 +7175,11 @@
       </c>
       <c r="C311" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D311" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="312">
@@ -8405,7 +8405,7 @@
     <row r="373">
       <c r="A373" s="8" t="inlineStr">
         <is>
-          <t>NQS-E1010</t>
+          <t>NQS-E1120</t>
         </is>
       </c>
       <c r="B373" s="8" t="inlineStr">
@@ -8415,11 +8415,11 @@
       </c>
       <c r="C373" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D373" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="374">
@@ -9645,7 +9645,7 @@
     <row r="435">
       <c r="A435" s="8" t="inlineStr">
         <is>
-          <t>EHF-E1010</t>
+          <t>EHF-E1120</t>
         </is>
       </c>
       <c r="B435" s="8" t="inlineStr">
@@ -9655,11 +9655,11 @@
       </c>
       <c r="C435" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D435" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="436">
@@ -10885,7 +10885,7 @@
     <row r="497">
       <c r="A497" s="8" t="inlineStr">
         <is>
-          <t>NMJ-E1010</t>
+          <t>NMJ-E1120</t>
         </is>
       </c>
       <c r="B497" s="8" t="inlineStr">
@@ -10895,11 +10895,11 @@
       </c>
       <c r="C497" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D497" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="498">
@@ -12125,7 +12125,7 @@
     <row r="559">
       <c r="A559" s="8" t="inlineStr">
         <is>
-          <t>HKA-E1010</t>
+          <t>HKA-E1120</t>
         </is>
       </c>
       <c r="B559" s="8" t="inlineStr">
@@ -12135,11 +12135,11 @@
       </c>
       <c r="C559" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D559" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="560">
@@ -13365,7 +13365,7 @@
     <row r="621">
       <c r="A621" s="8" t="inlineStr">
         <is>
-          <t>HMD-E1010</t>
+          <t>HMD-E1120</t>
         </is>
       </c>
       <c r="B621" s="8" t="inlineStr">
@@ -13375,11 +13375,11 @@
       </c>
       <c r="C621" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D621" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="622">
@@ -14605,7 +14605,7 @@
     <row r="683">
       <c r="A683" s="8" t="inlineStr">
         <is>
-          <t>EAB-E1010</t>
+          <t>EAB-E1120</t>
         </is>
       </c>
       <c r="B683" s="8" t="inlineStr">
@@ -14615,11 +14615,11 @@
       </c>
       <c r="C683" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D683" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="684">
@@ -15845,7 +15845,7 @@
     <row r="745">
       <c r="A745" s="8" t="inlineStr">
         <is>
-          <t>NHL-E1010</t>
+          <t>NHL-E1120</t>
         </is>
       </c>
       <c r="B745" s="8" t="inlineStr">
@@ -15855,11 +15855,11 @@
       </c>
       <c r="C745" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D745" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="746">
@@ -17085,7 +17085,7 @@
     <row r="807">
       <c r="A807" s="8" t="inlineStr">
         <is>
-          <t>NJF-E1010</t>
+          <t>NJF-E1120</t>
         </is>
       </c>
       <c r="B807" s="8" t="inlineStr">
@@ -17095,11 +17095,11 @@
       </c>
       <c r="C807" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D807" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="808">
@@ -18325,7 +18325,7 @@
     <row r="869">
       <c r="A869" s="8" t="inlineStr">
         <is>
-          <t>NQR-E1010</t>
+          <t>NQR-E1120</t>
         </is>
       </c>
       <c r="B869" s="8" t="inlineStr">
@@ -18335,11 +18335,11 @@
       </c>
       <c r="C869" s="8" t="inlineStr">
         <is>
-          <t>SS</t>
+          <t>FS</t>
         </is>
       </c>
       <c r="D869" s="8" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
     </row>
     <row r="870">
@@ -32304,10 +32304,10 @@
         <v/>
       </c>
       <c r="T28" s="20" t="n">
-        <v>46447</v>
+        <v>46509</v>
       </c>
       <c r="U28" s="20" t="n">
-        <v>46467</v>
+        <v>46520</v>
       </c>
       <c r="V28" s="8" t="n">
         <v>10</v>
@@ -32397,10 +32397,10 @@
         <v/>
       </c>
       <c r="T29" s="20" t="n">
-        <v>46468</v>
+        <v>46530</v>
       </c>
       <c r="U29" s="20" t="n">
-        <v>46488</v>
+        <v>46548</v>
       </c>
       <c r="V29" s="8" t="n">
         <v>15</v>
@@ -33141,10 +33141,10 @@
         <v/>
       </c>
       <c r="T37" s="20" t="n">
-        <v>46489</v>
+        <v>46551</v>
       </c>
       <c r="U37" s="20" t="n">
-        <v>46574</v>
+        <v>46629</v>
       </c>
       <c r="V37" s="8" t="n">
         <v>57</v>
@@ -33234,10 +33234,10 @@
         <v/>
       </c>
       <c r="T38" s="20" t="n">
-        <v>46547</v>
+        <v>46602</v>
       </c>
       <c r="U38" s="20" t="n">
-        <v>46609</v>
+        <v>46665</v>
       </c>
       <c r="V38" s="8" t="n">
         <v>45</v>
@@ -35652,10 +35652,10 @@
         <v/>
       </c>
       <c r="T64" s="20" t="n">
-        <v>46447</v>
+        <v>46509</v>
       </c>
       <c r="U64" s="20" t="n">
-        <v>46467</v>
+        <v>46520</v>
       </c>
       <c r="V64" s="8" t="n">
         <v>10</v>
@@ -35745,10 +35745,10 @@
         <v/>
       </c>
       <c r="T65" s="20" t="n">
-        <v>46468</v>
+        <v>46530</v>
       </c>
       <c r="U65" s="20" t="n">
-        <v>46488</v>
+        <v>46548</v>
       </c>
       <c r="V65" s="8" t="n">
         <v>15</v>
@@ -36489,10 +36489,10 @@
         <v/>
       </c>
       <c r="T73" s="20" t="n">
-        <v>46489</v>
+        <v>46551</v>
       </c>
       <c r="U73" s="20" t="n">
-        <v>46561</v>
+        <v>46616</v>
       </c>
       <c r="V73" s="8" t="n">
         <v>48</v>
@@ -36582,10 +36582,10 @@
         <v/>
       </c>
       <c r="T74" s="20" t="n">
-        <v>46539</v>
+        <v>46594</v>
       </c>
       <c r="U74" s="20" t="n">
-        <v>46589</v>
+        <v>46644</v>
       </c>
       <c r="V74" s="8" t="n">
         <v>37</v>
@@ -38907,10 +38907,10 @@
         <v/>
       </c>
       <c r="T99" s="20" t="n">
-        <v>46447</v>
+        <v>46509</v>
       </c>
       <c r="U99" s="20" t="n">
-        <v>46460</v>
+        <v>46513</v>
       </c>
       <c r="V99" s="8" t="n">
         <v>5</v>
@@ -39000,10 +39000,10 @@
         <v/>
       </c>
       <c r="T100" s="20" t="n">
-        <v>46461</v>
+        <v>46516</v>
       </c>
       <c r="U100" s="20" t="n">
-        <v>46474</v>
+        <v>46534</v>
       </c>
       <c r="V100" s="8" t="n">
         <v>10</v>
@@ -39744,10 +39744,10 @@
         <v/>
       </c>
       <c r="T108" s="20" t="n">
-        <v>46475</v>
+        <v>46537</v>
       </c>
       <c r="U108" s="20" t="n">
-        <v>46558</v>
+        <v>46611</v>
       </c>
       <c r="V108" s="8" t="n">
         <v>55</v>
@@ -39837,10 +39837,10 @@
         <v/>
       </c>
       <c r="T109" s="20" t="n">
-        <v>46531</v>
+        <v>46586</v>
       </c>
       <c r="U109" s="20" t="n">
-        <v>46589</v>
+        <v>46644</v>
       </c>
       <c r="V109" s="8" t="n">
         <v>43</v>
@@ -42162,10 +42162,10 @@
         <v/>
       </c>
       <c r="T134" s="20" t="n">
-        <v>46512</v>
+        <v>46569</v>
       </c>
       <c r="U134" s="20" t="n">
-        <v>46518</v>
+        <v>46575</v>
       </c>
       <c r="V134" s="8" t="n">
         <v>5</v>
@@ -42255,10 +42255,10 @@
         <v/>
       </c>
       <c r="T135" s="20" t="n">
-        <v>46519</v>
+        <v>46576</v>
       </c>
       <c r="U135" s="20" t="n">
-        <v>46539</v>
+        <v>46589</v>
       </c>
       <c r="V135" s="8" t="n">
         <v>10</v>
@@ -42999,10 +42999,10 @@
         <v/>
       </c>
       <c r="T143" s="20" t="n">
-        <v>46540</v>
+        <v>46590</v>
       </c>
       <c r="U143" s="20" t="n">
-        <v>46601</v>
+        <v>46651</v>
       </c>
       <c r="V143" s="8" t="n">
         <v>44</v>
@@ -43092,10 +43092,10 @@
         <v/>
       </c>
       <c r="T144" s="20" t="n">
-        <v>46580</v>
+        <v>46630</v>
       </c>
       <c r="U144" s="20" t="n">
-        <v>46628</v>
+        <v>46679</v>
       </c>
       <c r="V144" s="8" t="n">
         <v>35</v>
@@ -45417,10 +45417,10 @@
         <v/>
       </c>
       <c r="T169" s="20" t="n">
-        <v>46615</v>
+        <v>46677</v>
       </c>
       <c r="U169" s="20" t="n">
-        <v>46621</v>
+        <v>46681</v>
       </c>
       <c r="V169" s="8" t="n">
         <v>5</v>
@@ -45510,10 +45510,10 @@
         <v/>
       </c>
       <c r="T170" s="20" t="n">
-        <v>46622</v>
+        <v>46684</v>
       </c>
       <c r="U170" s="20" t="n">
-        <v>46635</v>
+        <v>46695</v>
       </c>
       <c r="V170" s="8" t="n">
         <v>10</v>
@@ -46254,10 +46254,10 @@
         <v/>
       </c>
       <c r="T178" s="20" t="n">
-        <v>46636</v>
+        <v>46698</v>
       </c>
       <c r="U178" s="20" t="n">
-        <v>46713</v>
+        <v>46772</v>
       </c>
       <c r="V178" s="8" t="n">
         <v>55</v>
@@ -46347,10 +46347,10 @@
         <v/>
       </c>
       <c r="T179" s="20" t="n">
-        <v>46686</v>
+        <v>46747</v>
       </c>
       <c r="U179" s="20" t="n">
-        <v>46744</v>
+        <v>46812</v>
       </c>
       <c r="V179" s="8" t="n">
         <v>43</v>
@@ -48672,10 +48672,10 @@
         <v/>
       </c>
       <c r="T204" s="20" t="n">
-        <v>46670</v>
+        <v>46733</v>
       </c>
       <c r="U204" s="20" t="n">
-        <v>46674</v>
+        <v>46737</v>
       </c>
       <c r="V204" s="8" t="n">
         <v>5</v>
@@ -48765,10 +48765,10 @@
         <v/>
       </c>
       <c r="T205" s="20" t="n">
-        <v>46677</v>
+        <v>46740</v>
       </c>
       <c r="U205" s="20" t="n">
-        <v>46688</v>
+        <v>46751</v>
       </c>
       <c r="V205" s="8" t="n">
         <v>10</v>
@@ -49509,10 +49509,10 @@
         <v/>
       </c>
       <c r="T213" s="20" t="n">
-        <v>46691</v>
+        <v>46754</v>
       </c>
       <c r="U213" s="20" t="n">
-        <v>46769</v>
+        <v>46839</v>
       </c>
       <c r="V213" s="8" t="n">
         <v>57</v>
@@ -49602,10 +49602,10 @@
         <v/>
       </c>
       <c r="T214" s="20" t="n">
-        <v>46742</v>
+        <v>46812</v>
       </c>
       <c r="U214" s="20" t="n">
-        <v>46811</v>
+        <v>46881</v>
       </c>
       <c r="V214" s="8" t="n">
         <v>45</v>
@@ -51927,10 +51927,10 @@
         <v/>
       </c>
       <c r="T239" s="20" t="n">
-        <v>46670</v>
+        <v>46733</v>
       </c>
       <c r="U239" s="20" t="n">
-        <v>46674</v>
+        <v>46737</v>
       </c>
       <c r="V239" s="8" t="n">
         <v>5</v>
@@ -52020,10 +52020,10 @@
         <v/>
       </c>
       <c r="T240" s="20" t="n">
-        <v>46677</v>
+        <v>46740</v>
       </c>
       <c r="U240" s="20" t="n">
-        <v>46688</v>
+        <v>46751</v>
       </c>
       <c r="V240" s="8" t="n">
         <v>10</v>
@@ -52764,10 +52764,10 @@
         <v/>
       </c>
       <c r="T248" s="20" t="n">
-        <v>46691</v>
+        <v>46754</v>
       </c>
       <c r="U248" s="20" t="n">
-        <v>46763</v>
+        <v>46833</v>
       </c>
       <c r="V248" s="8" t="n">
         <v>53</v>
@@ -52857,10 +52857,10 @@
         <v/>
       </c>
       <c r="T249" s="20" t="n">
-        <v>46737</v>
+        <v>46800</v>
       </c>
       <c r="U249" s="20" t="n">
-        <v>46793</v>
+        <v>46863</v>
       </c>
       <c r="V249" s="8" t="n">
         <v>41</v>
@@ -55182,10 +55182,10 @@
         <v/>
       </c>
       <c r="T274" s="20" t="n">
-        <v>46716</v>
+        <v>46782</v>
       </c>
       <c r="U274" s="20" t="n">
-        <v>46722</v>
+        <v>46786</v>
       </c>
       <c r="V274" s="8" t="n">
         <v>5</v>
@@ -55275,10 +55275,10 @@
         <v/>
       </c>
       <c r="T275" s="20" t="n">
-        <v>46723</v>
+        <v>46789</v>
       </c>
       <c r="U275" s="20" t="n">
-        <v>46736</v>
+        <v>46800</v>
       </c>
       <c r="V275" s="8" t="n">
         <v>10</v>
@@ -56019,10 +56019,10 @@
         <v/>
       </c>
       <c r="T283" s="20" t="n">
-        <v>46737</v>
+        <v>46810</v>
       </c>
       <c r="U283" s="20" t="n">
-        <v>46824</v>
+        <v>46895</v>
       </c>
       <c r="V283" s="8" t="n">
         <v>57</v>
@@ -56112,10 +56112,10 @@
         <v/>
       </c>
       <c r="T284" s="20" t="n">
-        <v>46790</v>
+        <v>46861</v>
       </c>
       <c r="U284" s="20" t="n">
-        <v>46859</v>
+        <v>46930</v>
       </c>
       <c r="V284" s="8" t="n">
         <v>45</v>
@@ -58437,10 +58437,10 @@
         <v/>
       </c>
       <c r="T309" s="20" t="n">
-        <v>46842</v>
+        <v>46898</v>
       </c>
       <c r="U309" s="20" t="n">
-        <v>46848</v>
+        <v>46904</v>
       </c>
       <c r="V309" s="8" t="n">
         <v>5</v>
@@ -58530,10 +58530,10 @@
         <v/>
       </c>
       <c r="T310" s="20" t="n">
-        <v>46849</v>
+        <v>46905</v>
       </c>
       <c r="U310" s="20" t="n">
-        <v>46862</v>
+        <v>46918</v>
       </c>
       <c r="V310" s="8" t="n">
         <v>10</v>
@@ -59274,10 +59274,10 @@
         <v/>
       </c>
       <c r="T318" s="20" t="n">
-        <v>46863</v>
+        <v>46919</v>
       </c>
       <c r="U318" s="20" t="n">
-        <v>46904</v>
+        <v>46953</v>
       </c>
       <c r="V318" s="8" t="n">
         <v>25</v>
@@ -59367,10 +59367,10 @@
         <v/>
       </c>
       <c r="T319" s="20" t="n">
-        <v>46894</v>
+        <v>46943</v>
       </c>
       <c r="U319" s="20" t="n">
-        <v>46919</v>
+        <v>46968</v>
       </c>
       <c r="V319" s="8" t="n">
         <v>20</v>
@@ -61692,10 +61692,10 @@
         <v/>
       </c>
       <c r="T344" s="20" t="n">
-        <v>46842</v>
+        <v>46898</v>
       </c>
       <c r="U344" s="20" t="n">
-        <v>46848</v>
+        <v>46904</v>
       </c>
       <c r="V344" s="8" t="n">
         <v>5</v>
@@ -61785,10 +61785,10 @@
         <v/>
       </c>
       <c r="T345" s="20" t="n">
-        <v>46849</v>
+        <v>46905</v>
       </c>
       <c r="U345" s="20" t="n">
-        <v>46862</v>
+        <v>46918</v>
       </c>
       <c r="V345" s="8" t="n">
         <v>10</v>
@@ -62529,10 +62529,10 @@
         <v/>
       </c>
       <c r="T353" s="20" t="n">
-        <v>46863</v>
+        <v>46919</v>
       </c>
       <c r="U353" s="20" t="n">
-        <v>46912</v>
+        <v>46961</v>
       </c>
       <c r="V353" s="8" t="n">
         <v>31</v>
@@ -62622,10 +62622,10 @@
         <v/>
       </c>
       <c r="T354" s="20" t="n">
-        <v>46898</v>
+        <v>46947</v>
       </c>
       <c r="U354" s="20" t="n">
-        <v>46931</v>
+        <v>46980</v>
       </c>
       <c r="V354" s="8" t="n">
         <v>24</v>
@@ -64947,10 +64947,10 @@
         <v/>
       </c>
       <c r="T379" s="20" t="n">
-        <v>46897</v>
+        <v>46954</v>
       </c>
       <c r="U379" s="20" t="n">
-        <v>46903</v>
+        <v>46960</v>
       </c>
       <c r="V379" s="8" t="n">
         <v>5</v>
@@ -65040,10 +65040,10 @@
         <v/>
       </c>
       <c r="T380" s="20" t="n">
-        <v>46904</v>
+        <v>46961</v>
       </c>
       <c r="U380" s="20" t="n">
-        <v>46917</v>
+        <v>46974</v>
       </c>
       <c r="V380" s="8" t="n">
         <v>10</v>
@@ -65784,10 +65784,10 @@
         <v/>
       </c>
       <c r="T388" s="20" t="n">
-        <v>46918</v>
+        <v>46975</v>
       </c>
       <c r="U388" s="20" t="n">
-        <v>46967</v>
+        <v>47024</v>
       </c>
       <c r="V388" s="8" t="n">
         <v>36</v>
@@ -65877,10 +65877,10 @@
         <v/>
       </c>
       <c r="T389" s="20" t="n">
-        <v>46951</v>
+        <v>47008</v>
       </c>
       <c r="U389" s="20" t="n">
-        <v>46988</v>
+        <v>47045</v>
       </c>
       <c r="V389" s="8" t="n">
         <v>28</v>
@@ -68202,10 +68202,10 @@
         <v/>
       </c>
       <c r="T414" s="20" t="n">
-        <v>46922</v>
+        <v>46978</v>
       </c>
       <c r="U414" s="20" t="n">
-        <v>46926</v>
+        <v>46982</v>
       </c>
       <c r="V414" s="8" t="n">
         <v>5</v>
@@ -68295,10 +68295,10 @@
         <v/>
       </c>
       <c r="T415" s="20" t="n">
-        <v>46929</v>
+        <v>46985</v>
       </c>
       <c r="U415" s="20" t="n">
-        <v>46940</v>
+        <v>46996</v>
       </c>
       <c r="V415" s="8" t="n">
         <v>10</v>
@@ -69039,10 +69039,10 @@
         <v/>
       </c>
       <c r="T423" s="20" t="n">
-        <v>46943</v>
+        <v>46999</v>
       </c>
       <c r="U423" s="20" t="n">
-        <v>47021</v>
+        <v>47077</v>
       </c>
       <c r="V423" s="8" t="n">
         <v>57</v>
@@ -69132,10 +69132,10 @@
         <v/>
       </c>
       <c r="T424" s="20" t="n">
-        <v>46994</v>
+        <v>47050</v>
       </c>
       <c r="U424" s="20" t="n">
-        <v>47056</v>
+        <v>47112</v>
       </c>
       <c r="V424" s="8" t="n">
         <v>45</v>
@@ -71457,10 +71457,10 @@
         <v/>
       </c>
       <c r="T449" s="20" t="n">
-        <v>46993</v>
+        <v>47055</v>
       </c>
       <c r="U449" s="20" t="n">
-        <v>46999</v>
+        <v>47059</v>
       </c>
       <c r="V449" s="8" t="n">
         <v>5</v>
@@ -71550,10 +71550,10 @@
         <v/>
       </c>
       <c r="T450" s="20" t="n">
-        <v>47000</v>
+        <v>47062</v>
       </c>
       <c r="U450" s="20" t="n">
-        <v>47013</v>
+        <v>47073</v>
       </c>
       <c r="V450" s="8" t="n">
         <v>10</v>
@@ -72294,10 +72294,10 @@
         <v/>
       </c>
       <c r="T458" s="20" t="n">
-        <v>47014</v>
+        <v>47076</v>
       </c>
       <c r="U458" s="20" t="n">
-        <v>47092</v>
+        <v>47154</v>
       </c>
       <c r="V458" s="8" t="n">
         <v>57</v>
@@ -72387,10 +72387,10 @@
         <v/>
       </c>
       <c r="T459" s="20" t="n">
-        <v>47065</v>
+        <v>47127</v>
       </c>
       <c r="U459" s="20" t="n">
-        <v>47127</v>
+        <v>47197</v>
       </c>
       <c r="V459" s="8" t="n">
         <v>45</v>
@@ -74712,10 +74712,10 @@
         <v/>
       </c>
       <c r="T484" s="20" t="n">
-        <v>47041</v>
+        <v>47104</v>
       </c>
       <c r="U484" s="20" t="n">
-        <v>47045</v>
+        <v>47108</v>
       </c>
       <c r="V484" s="8" t="n">
         <v>5</v>
@@ -74805,10 +74805,10 @@
         <v/>
       </c>
       <c r="T485" s="20" t="n">
-        <v>47048</v>
+        <v>47111</v>
       </c>
       <c r="U485" s="20" t="n">
-        <v>47059</v>
+        <v>47122</v>
       </c>
       <c r="V485" s="8" t="n">
         <v>10</v>
@@ -75549,10 +75549,10 @@
         <v/>
       </c>
       <c r="T493" s="20" t="n">
-        <v>47062</v>
+        <v>47125</v>
       </c>
       <c r="U493" s="20" t="n">
-        <v>47140</v>
+        <v>47211</v>
       </c>
       <c r="V493" s="8" t="n">
         <v>57</v>
@@ -75642,10 +75642,10 @@
         <v/>
       </c>
       <c r="T494" s="20" t="n">
-        <v>47113</v>
+        <v>47184</v>
       </c>
       <c r="U494" s="20" t="n">
-        <v>47183</v>
+        <v>47253</v>
       </c>
       <c r="V494" s="8" t="n">
         <v>45</v>
@@ -77169,7 +77169,7 @@
         <v>46447</v>
       </c>
       <c r="B8" s="9" t="n">
-        <v>1206616.967042765</v>
+        <v>1149268.960982159</v>
       </c>
       <c r="C8" s="9">
         <f>SUM(B$4:B8)</f>
@@ -77180,7 +77180,7 @@
         <v/>
       </c>
       <c r="E8" s="10" t="n">
-        <v>0.01491215547197903</v>
+        <v>0.009865185775009288</v>
       </c>
       <c r="F8" s="23">
         <f>SUM(E$4:E8)</f>
@@ -77192,7 +77192,7 @@
         <v>46478</v>
       </c>
       <c r="B9" s="9" t="n">
-        <v>1736189.828750072</v>
+        <v>1628197.492027584</v>
       </c>
       <c r="C9" s="9">
         <f>SUM(B$4:B9)</f>
@@ -77203,7 +77203,7 @@
         <v/>
       </c>
       <c r="E9" s="10" t="n">
-        <v>0.01920797853359233</v>
+        <v>0.01287862486533075</v>
       </c>
       <c r="F9" s="23">
         <f>SUM(E$4:E9)</f>
@@ -77215,7 +77215,7 @@
         <v>46508</v>
       </c>
       <c r="B10" s="9" t="n">
-        <v>1435486.418335914</v>
+        <v>1359773.798666298</v>
       </c>
       <c r="C10" s="9">
         <f>SUM(B$4:B10)</f>
@@ -77226,7 +77226,7 @@
         <v/>
       </c>
       <c r="E10" s="10" t="n">
-        <v>0.03127697796773721</v>
+        <v>0.02678590646167296</v>
       </c>
       <c r="F10" s="23">
         <f>SUM(E$4:E10)</f>
@@ -77238,7 +77238,7 @@
         <v>46539</v>
       </c>
       <c r="B11" s="9" t="n">
-        <v>1953908.69113037</v>
+        <v>1796308.819662572</v>
       </c>
       <c r="C11" s="9">
         <f>SUM(B$4:B11)</f>
@@ -77249,7 +77249,7 @@
         <v/>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0.0451129400784422</v>
+        <v>0.03464160657540269</v>
       </c>
       <c r="F11" s="23">
         <f>SUM(E$4:E11)</f>
@@ -77261,7 +77261,7 @@
         <v>46569</v>
       </c>
       <c r="B12" s="9" t="n">
-        <v>1301536.665192205</v>
+        <v>1303669.89269185</v>
       </c>
       <c r="C12" s="9">
         <f>SUM(B$4:B12)</f>
@@ -77272,7 +77272,7 @@
         <v/>
       </c>
       <c r="E12" s="10" t="n">
-        <v>0.04210792094747215</v>
+        <v>0.0423125577926599</v>
       </c>
       <c r="F12" s="23">
         <f>SUM(E$4:E12)</f>
@@ -77284,7 +77284,7 @@
         <v>46600</v>
       </c>
       <c r="B13" s="9" t="n">
-        <v>1434567.071153576</v>
+        <v>1625994.299509653</v>
       </c>
       <c r="C13" s="9">
         <f>SUM(B$4:B13)</f>
@@ -77295,7 +77295,7 @@
         <v/>
       </c>
       <c r="E13" s="10" t="n">
-        <v>0.04062566597934238</v>
+        <v>0.05127385094940848</v>
       </c>
       <c r="F13" s="23">
         <f>SUM(E$4:E13)</f>
@@ -77307,7 +77307,7 @@
         <v>46631</v>
       </c>
       <c r="B14" s="9" t="n">
-        <v>1651510.041674334</v>
+        <v>1766294.476016181</v>
       </c>
       <c r="C14" s="9">
         <f>SUM(B$4:B14)</f>
@@ -77318,7 +77318,7 @@
         <v/>
       </c>
       <c r="E14" s="10" t="n">
-        <v>0.03596624505406881</v>
+        <v>0.04624741568241361</v>
       </c>
       <c r="F14" s="23">
         <f>SUM(E$4:E14)</f>
@@ -77330,7 +77330,7 @@
         <v>46661</v>
       </c>
       <c r="B15" s="9" t="n">
-        <v>1729273.516660846</v>
+        <v>1682512.409514225</v>
       </c>
       <c r="C15" s="9">
         <f>SUM(B$4:B15)</f>
@@ -77341,7 +77341,7 @@
         <v/>
       </c>
       <c r="E15" s="10" t="n">
-        <v>0.03817357021076049</v>
+        <v>0.03804258329654849</v>
       </c>
       <c r="F15" s="23">
         <f>SUM(E$4:E15)</f>
@@ -77353,7 +77353,7 @@
         <v>46692</v>
       </c>
       <c r="B16" s="9" t="n">
-        <v>2392620.12902667</v>
+        <v>2266493.398056921</v>
       </c>
       <c r="C16" s="9">
         <f>SUM(B$4:B16)</f>
@@ -77364,7 +77364,7 @@
         <v/>
       </c>
       <c r="E16" s="10" t="n">
-        <v>0.04403924707643078</v>
+        <v>0.040261234551001</v>
       </c>
       <c r="F16" s="23">
         <f>SUM(E$4:E16)</f>
@@ -77376,7 +77376,7 @@
         <v>46722</v>
       </c>
       <c r="B17" s="9" t="n">
-        <v>2014067.062838126</v>
+        <v>1919790.529655363</v>
       </c>
       <c r="C17" s="9">
         <f>SUM(B$4:B17)</f>
@@ -77387,7 +77387,7 @@
         <v/>
       </c>
       <c r="E17" s="10" t="n">
-        <v>0.0460688563673353</v>
+        <v>0.04396941864266432</v>
       </c>
       <c r="F17" s="23">
         <f>SUM(E$4:E17)</f>
@@ -77399,7 +77399,7 @@
         <v>46753</v>
       </c>
       <c r="B18" s="9" t="n">
-        <v>2254093.084222251</v>
+        <v>2252018.442109223</v>
       </c>
       <c r="C18" s="9">
         <f>SUM(B$4:B18)</f>
@@ -77410,7 +77410,7 @@
         <v/>
       </c>
       <c r="E18" s="10" t="n">
-        <v>0.04421882690995473</v>
+        <v>0.04414193284532374</v>
       </c>
       <c r="F18" s="23">
         <f>SUM(E$4:E18)</f>
@@ -77422,7 +77422,7 @@
         <v>46784</v>
       </c>
       <c r="B19" s="9" t="n">
-        <v>1547362.1648266</v>
+        <v>1577811.5641617</v>
       </c>
       <c r="C19" s="9">
         <f>SUM(B$4:B19)</f>
@@ -77433,7 +77433,7 @@
         <v/>
       </c>
       <c r="E19" s="10" t="n">
-        <v>0.03253845171996104</v>
+        <v>0.03387268475375258</v>
       </c>
       <c r="F19" s="23">
         <f>SUM(E$4:E19)</f>
@@ -77445,7 +77445,7 @@
         <v>46813</v>
       </c>
       <c r="B20" s="9" t="n">
-        <v>2628648.261655338</v>
+        <v>2762045.924319129</v>
       </c>
       <c r="C20" s="9">
         <f>SUM(B$4:B20)</f>
@@ -77456,7 +77456,7 @@
         <v/>
       </c>
       <c r="E20" s="10" t="n">
-        <v>0.04529831496648301</v>
+        <v>0.04891604069128763</v>
       </c>
       <c r="F20" s="23">
         <f>SUM(E$4:E20)</f>
@@ -77468,7 +77468,7 @@
         <v>46844</v>
       </c>
       <c r="B21" s="9" t="n">
-        <v>3312454.656340744</v>
+        <v>3379027.264459413</v>
       </c>
       <c r="C21" s="9">
         <f>SUM(B$4:B21)</f>
@@ -77479,7 +77479,7 @@
         <v/>
       </c>
       <c r="E21" s="10" t="n">
-        <v>0.05053857981140839</v>
+        <v>0.04714948391141734</v>
       </c>
       <c r="F21" s="23">
         <f>SUM(E$4:E21)</f>
@@ -77491,7 +77491,7 @@
         <v>46874</v>
       </c>
       <c r="B22" s="9" t="n">
-        <v>2525511.031383557</v>
+        <v>2513138.951734432</v>
       </c>
       <c r="C22" s="9">
         <f>SUM(B$4:B22)</f>
@@ -77502,7 +77502,7 @@
         <v/>
       </c>
       <c r="E22" s="10" t="n">
-        <v>0.04726796061307757</v>
+        <v>0.04005261921522792</v>
       </c>
       <c r="F22" s="23">
         <f>SUM(E$4:E22)</f>
@@ -77514,7 +77514,7 @@
         <v>46905</v>
       </c>
       <c r="B23" s="9" t="n">
-        <v>2725504.452635161</v>
+        <v>2704699.365968495</v>
       </c>
       <c r="C23" s="9">
         <f>SUM(B$4:B23)</f>
@@ -77525,7 +77525,7 @@
         <v/>
       </c>
       <c r="E23" s="10" t="n">
-        <v>0.05254287047177084</v>
+        <v>0.05173817961155595</v>
       </c>
       <c r="F23" s="23">
         <f>SUM(E$4:E23)</f>
@@ -77537,7 +77537,7 @@
         <v>46935</v>
       </c>
       <c r="B24" s="9" t="n">
-        <v>2208849.678818159</v>
+        <v>2217277.2476068</v>
       </c>
       <c r="C24" s="9">
         <f>SUM(B$4:B24)</f>
@@ -77548,7 +77548,7 @@
         <v/>
       </c>
       <c r="E24" s="10" t="n">
-        <v>0.03938885435468486</v>
+        <v>0.04932846789795158</v>
       </c>
       <c r="F24" s="23">
         <f>SUM(E$4:E24)</f>
@@ -77560,7 +77560,7 @@
         <v>46966</v>
       </c>
       <c r="B25" s="9" t="n">
-        <v>1806364.315503699</v>
+        <v>1794009.798878804</v>
       </c>
       <c r="C25" s="9">
         <f>SUM(B$4:B25)</f>
@@ -77571,7 +77571,7 @@
         <v/>
       </c>
       <c r="E25" s="10" t="n">
-        <v>0.03808806098869292</v>
+        <v>0.04022412844901042</v>
       </c>
       <c r="F25" s="23">
         <f>SUM(E$4:E25)</f>
@@ -77583,7 +77583,7 @@
         <v>46997</v>
       </c>
       <c r="B26" s="9" t="n">
-        <v>1154977.748705478</v>
+        <v>1146711.540434802</v>
       </c>
       <c r="C26" s="9">
         <f>SUM(B$4:B26)</f>
@@ -77594,7 +77594,7 @@
         <v/>
       </c>
       <c r="E26" s="10" t="n">
-        <v>0.02757175335283647</v>
+        <v>0.02698557164857578</v>
       </c>
       <c r="F26" s="23">
         <f>SUM(E$4:E26)</f>
@@ -77606,7 +77606,7 @@
         <v>47027</v>
       </c>
       <c r="B27" s="9" t="n">
-        <v>1409882.753788003</v>
+        <v>1391672.180772132</v>
       </c>
       <c r="C27" s="9">
         <f>SUM(B$4:B27)</f>
@@ -77617,7 +77617,7 @@
         <v/>
       </c>
       <c r="E27" s="10" t="n">
-        <v>0.03310759739754984</v>
+        <v>0.03215077325385727</v>
       </c>
       <c r="F27" s="23">
         <f>SUM(E$4:E27)</f>
@@ -77629,7 +77629,7 @@
         <v>47058</v>
       </c>
       <c r="B28" s="9" t="n">
-        <v>1772895.198802991</v>
+        <v>1762471.077165564</v>
       </c>
       <c r="C28" s="9">
         <f>SUM(B$4:B28)</f>
@@ -77640,7 +77640,7 @@
         <v/>
       </c>
       <c r="E28" s="10" t="n">
-        <v>0.03376821548806752</v>
+        <v>0.03381267162841844</v>
       </c>
       <c r="F28" s="23">
         <f>SUM(E$4:E28)</f>
@@ -77652,7 +77652,7 @@
         <v>47088</v>
       </c>
       <c r="B29" s="9" t="n">
-        <v>1657383.011696295</v>
+        <v>1652866.22105302</v>
       </c>
       <c r="C29" s="9">
         <f>SUM(B$4:B29)</f>
@@ -77663,7 +77663,7 @@
         <v/>
       </c>
       <c r="E29" s="10" t="n">
-        <v>0.03204975435021504</v>
+        <v>0.03240318125079989</v>
       </c>
       <c r="F29" s="23">
         <f>SUM(E$4:E29)</f>
@@ -77675,7 +77675,7 @@
         <v>47119</v>
       </c>
       <c r="B30" s="9" t="n">
-        <v>1544621.848645296</v>
+        <v>1573399.130516641</v>
       </c>
       <c r="C30" s="9">
         <f>SUM(B$4:B30)</f>
@@ -77686,7 +77686,7 @@
         <v/>
       </c>
       <c r="E30" s="10" t="n">
-        <v>0.03045369595671562</v>
+        <v>0.03158243279882086</v>
       </c>
       <c r="F30" s="23">
         <f>SUM(E$4:E30)</f>
@@ -77698,7 +77698,7 @@
         <v>47150</v>
       </c>
       <c r="B31" s="9" t="n">
-        <v>1373489.649442756</v>
+        <v>1404924.737162054</v>
       </c>
       <c r="C31" s="9">
         <f>SUM(B$4:B31)</f>
@@ -77709,7 +77709,7 @@
         <v/>
       </c>
       <c r="E31" s="10" t="n">
-        <v>0.02086956190322678</v>
+        <v>0.02189683675702795</v>
       </c>
       <c r="F31" s="23">
         <f>SUM(E$4:E31)</f>
@@ -77721,7 +77721,7 @@
         <v>47178</v>
       </c>
       <c r="B32" s="9" t="n">
-        <v>1078569.686926963</v>
+        <v>1167993.26587433</v>
       </c>
       <c r="C32" s="9">
         <f>SUM(B$4:B32)</f>
@@ -77732,7 +77732,7 @@
         <v/>
       </c>
       <c r="E32" s="10" t="n">
-        <v>0.02009785311910314</v>
+        <v>0.02294207534132536</v>
       </c>
       <c r="F32" s="23">
         <f>SUM(E$4:E32)</f>
@@ -77744,7 +77744,7 @@
         <v>47209</v>
       </c>
       <c r="B33" s="9" t="n">
-        <v>714788.0124320129</v>
+        <v>752189.6030752873</v>
       </c>
       <c r="C33" s="9">
         <f>SUM(B$4:B33)</f>
@@ -77755,7 +77755,7 @@
         <v/>
       </c>
       <c r="E33" s="10" t="n">
-        <v>0.01467548174048175</v>
+        <v>0.01584903729603731</v>
       </c>
       <c r="F33" s="23">
         <f>SUM(E$4:E33)</f>
@@ -77767,7 +77767,7 @@
         <v>47239</v>
       </c>
       <c r="B34" s="9" t="n">
-        <v>923106.7743145761</v>
+        <v>943718.3298701313</v>
       </c>
       <c r="C34" s="9">
         <f>SUM(B$4:B34)</f>
@@ -77778,7 +77778,7 @@
         <v/>
       </c>
       <c r="E34" s="10" t="n">
-        <v>0.01448861516261515</v>
+        <v>0.01513150405150403</v>
       </c>
       <c r="F34" s="23">
         <f>SUM(E$4:E34)</f>

</xml_diff>